<commit_message>
docs: extend qa cases and bug table
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -294,6 +294,515 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adm:ord:* меняет чужие заказы без проверки tenant</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Владелец магазина B узнаёт ID заказа магазина A.
+2. Нажимает adm:ord:accept:&lt;id&gt;.
+Actual Result: заказ мутирует до проверки принадлежности.
+Expected Result: проверка tenant до applyOrderEvent, ответ «Заказ не найден».
+Fix: loadOwnedOrder guard + тест.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">my:view/cancel/pay без фильтра tenant</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Один telegramId в двух магазинах.
+2. Открыть чужой заказ через my:view.
+Actual Result: заказ другого магазина виден.
+Expected Result: фильтр orders.tenantId + customers.tenantId.
+Fix: добавлены фильтры + тест.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Двойной pd:yes переписывает дату принятого заказа</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Владелец предлагает дату.
+2. Клиент дважды жмёт «Подходит».
+Actual Result: вторая запись без проверки.
+Expected Result: атомарный acceptProposedDate, второй вызов отклонён.
+Fix: сервис acceptProposedDate + тест.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adm:ord:pd пишет недоступную дату</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Предложить дату через forged callback на закрытый день.
+Actual Result: proposedDate записан без проверки.
+Expected Result: проверка getDateAvailability, ответ «Дата уже недоступна».
+Fix: проверка + тест.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Повторная оплата не пересоздаёт джобы</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Принять заказ, отклонить чек.
+Actual Result: старые done-джобы блокируют новые runAt.
+Expected Result: upsert runAt/pending/attempts при re-entry.
+Fix: onConflictDoUpdate + тест.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Двойной чек оставляет orphan-запись</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Прислать чек дважды быстро.
+Actual Result: insert чека до transition, orphan при ILLEGAL_TRANSITION.
+Expected Result: сначала transition, потом insert.
+Fix: переупорядочено + тест.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Доставка без адреса проходит</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Оформить доставку без адреса.
+Actual Result: заказ создан.
+Expected Result: BAD_ADDRESS в createOrder и chk:submit.
+Fix: проверка + контракт v1.19 + тест.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Телефон без имени ведёт в тупик</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Ввести только телефон в checkout.contact.
+Actual Result: submit падает с incomplete.
+Expected Result: просьба указать имя.
+Fix: contactNameMissing + тест.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Пустой выбор опций занижает цену</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Создать заказ с optionIds=[] на товар с опциями.
+Actual Result: цена без доплат.
+Expected Result: BAD_OPTIONS при неполном выборе.
+Fix: строгая валидация + контракт v1.20 + тест.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Заблокированный клиент оформляет заказ</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Заблокировать клиента.
+2. Начать оформление через каталог.
+Actual Result: заказ создан.
+Expected Result: CUSTOMER_BLOCKED в createOrder и chk:start.
+Fix: проверка + контракт v1.21 + тест.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Голосовые сообщения не пересылаются</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Клиент отправляет voice.
+Actual Result: сообщение теряется.
+Expected Result: relay владельцу (контракт 8.4).
+Fix: message:voice handler + тест.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLOCKED без уведомления владельца</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Клиент блокирует бота.
+2. Джоб падает.
+Actual Result: флаг ставится, владелец не знает.
+Expected Result: sendCustomerMessage уведомляет один раз.
+Fix: центральный helper + тест.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Текст relay спамит двумя сообщениями</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Клиент пишет текст.
+Actual Result: header + copy = 2 сообщения владельцу.
+Expected Result: одно сообщение шапка+текст.
+Fix: объединено + тест.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minor</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ретраи джобов: 2 вместо 3</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Джоб падает 3 раза.
+Actual Result: failed после 2 ретраев, 1800s никогда.
+Expected Result: 3 ретрая по контракту 8.2.
+Fix: &lt;= + тест.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Major</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: antispam revival rule and critical bug log
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -803,6 +803,43 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Антиспам блокирует все включая /start после ~20 действий</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. Активно проходить оформление (клики + тексты + фото).
+2. Набрать &gt;20 апдейтов за минуту.
+Actual Result: 5 минут тишины, /start не оживляет.
+Expected Result: /start и /menu всегда работают и сбрасывают лимит; блоки логируются.
+Fix: exemption revival-команд + warn-лог + лимит комментария + тесты.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: log session race bug and status
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -840,6 +840,42 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Альбом фото считается как одно: гонка сессии</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STR:
+1. В checkout.photos отправить альбом из 5 фото разом.
+Actual Result: в черновике оставалось 1 фото (last writer wins при параллельных апдейтах).
+Expected Result: все фото засчитаны.
+Fix: serializeMiddleware — строгая последовательность апдейтов чата + регрессионный тест (без фикса падает).</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(contracts): tech v1.28 and qa bug resolutions
Contract: SendOpts replyKeyboard/removeKeyboard, SessionData.contactKbMsgId. QA: reconcile bug IDs 24-28 from Numbers, add resolutions, log 29-32.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -1,61 +1,462 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Bugs" sheetId="1" r:id="rId1"/>
+    <sheet name="Bugs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Summary</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Description</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Priority</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Severity</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attachments</t>
+          <t>Attachments</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner menu: «Заказы» не открывает список</t>
+          <t>Owner menu: «Заказы» не открывает список</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Открыть owner menu.
 2. Нажать «Заказы».
 Actual Result: обработчик `adm:ord:list` отсутствует, список не открывается.
@@ -65,34 +466,29 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner menu: «Как видит клиент» не обрабатывается</t>
+          <t>Owner menu: «Как видит клиент» не обрабатывается</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Открыть owner menu.
 2. Нажать «Как видит клиент».
 Actual Result: обработчик `adm:preview` отсутствует, экран не открывается.
@@ -101,34 +497,29 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Superadmin-owner видит клиентский `/menu` вместо owner-screen</t>
+          <t>Superadmin-owner видит клиентский `/menu` вместо owner-screen</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Установить токен магазина.
 2. Открыть `/menu` пользователем, который является owner и superadmin.
 Actual Result: roleMiddleware выставляет `superadmin`, `/menu` уходит в клиентскую ветку, owner-разделы скрыты.
@@ -137,34 +528,29 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нет кнопки «Назад» на нескольких owner-экранах</t>
+          <t>Нет кнопки «Назад» на нескольких owner-экранах</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Открыть Settings.
 2. Переключить «Перегруз».
 Actual Result: сообщение об переключении приходит без клавиатуры возврата.
@@ -173,34 +559,29 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minor</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Minor</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нет прямого перехода «Написать клиенту» из карточки заказа</t>
+          <t>Нет прямого перехода «Написать клиенту» из карточки заказа</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Открыть заказ.
 2. Найти кнопку «Написать клиенту».
 Actual Result: в коде контракта `adm:ord:msg` нет, кнопка не отображается.
@@ -209,34 +590,29 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep-link `/deleteme` не обрабатывается</t>
+          <t>Deep-link `/deleteme` не обрабатывается</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Отправить `/deleteme`.
 Actual Result: message:text relay перехватывает команду и не вызывает deleteme-handler.
 Expected Result: удаление/обезличивание пользователя.</t>
@@ -244,34 +620,29 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAQ label display style не единый</t>
+          <t>FAQ label display style не единый</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Открыть owner menu.
 2. Посмотреть кнопку FAQ.
 Actual Result: в owner menu было `FAQ`, в других местах «Вопросы и ответы».
@@ -280,34 +651,29 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minor</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Minor</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">adm:ord:* меняет чужие заказы без проверки tenant</t>
+          <t>adm:ord:* меняет чужие заказы без проверки tenant</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Владелец магазина B узнаёт ID заказа магазина A.
 2. Нажимает adm:ord:accept:&lt;id&gt;.
 Actual Result: заказ мутирует до проверки принадлежности.
@@ -317,34 +683,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">my:view/cancel/pay без фильтра tenant</t>
+          <t>my:view/cancel/pay без фильтра tenant</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Один telegramId в двух магазинах.
 2. Открыть чужой заказ через my:view.
 Actual Result: заказ другого магазина виден.
@@ -354,34 +715,29 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Двойной pd:yes переписывает дату принятого заказа</t>
+          <t>Двойной pd:yes переписывает дату принятого заказа</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Владелец предлагает дату.
 2. Клиент дважды жмёт «Подходит».
 Actual Result: вторая запись без проверки.
@@ -391,34 +747,29 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">adm:ord:pd пишет недоступную дату</t>
+          <t>adm:ord:pd пишет недоступную дату</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Предложить дату через forged callback на закрытый день.
 Actual Result: proposedDate записан без проверки.
 Expected Result: проверка getDateAvailability, ответ «Дата уже недоступна».
@@ -427,34 +778,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Повторная оплата не пересоздаёт джобы</t>
+          <t>Повторная оплата не пересоздаёт джобы</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Принять заказ, отклонить чек.
 Actual Result: старые done-джобы блокируют новые runAt.
 Expected Result: upsert runAt/pending/attempts при re-entry.
@@ -463,34 +809,29 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Двойной чек оставляет orphan-запись</t>
+          <t>Двойной чек оставляет orphan-запись</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Прислать чек дважды быстро.
 Actual Result: insert чека до transition, orphan при ILLEGAL_TRANSITION.
 Expected Result: сначала transition, потом insert.
@@ -499,34 +840,29 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">14</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Доставка без адреса проходит</t>
+          <t>Доставка без адреса проходит</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Оформить доставку без адреса.
 Actual Result: заказ создан.
 Expected Result: BAD_ADDRESS в createOrder и chk:submit.
@@ -535,34 +871,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Телефон без имени ведёт в тупик</t>
+          <t>Телефон без имени ведёт в тупик</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Ввести только телефон в checkout.contact.
 Actual Result: submit падает с incomplete.
 Expected Result: просьба указать имя.
@@ -571,34 +902,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minor</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Minor</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">16</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пустой выбор опций занижает цену</t>
+          <t>Пустой выбор опций занижает цену</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Создать заказ с optionIds=[] на товар с опциями.
 Actual Result: цена без доплат.
 Expected Result: BAD_OPTIONS при неполном выборе.
@@ -607,34 +933,29 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">17</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заблокированный клиент оформляет заказ</t>
+          <t>Заблокированный клиент оформляет заказ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Заблокировать клиента.
 2. Начать оформление через каталог.
 Actual Result: заказ создан.
@@ -644,34 +965,29 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">18</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Голосовые сообщения не пересылаются</t>
+          <t>Голосовые сообщения не пересылаются</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Клиент отправляет voice.
 Actual Result: сообщение теряется.
 Expected Result: relay владельцу (контракт 8.4).
@@ -680,34 +996,29 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">19</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCKED без уведомления владельца</t>
+          <t>BLOCKED без уведомления владельца</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Клиент блокирует бота.
 2. Джоб падает.
 Actual Result: флаг ставится, владелец не знает.
@@ -717,34 +1028,29 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Текст relay спамит двумя сообщениями</t>
+          <t>Текст relay спамит двумя сообщениями</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Клиент пишет текст.
 Actual Result: header + copy = 2 сообщения владельцу.
 Expected Result: одно сообщение шапка+текст.
@@ -753,34 +1059,29 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minor</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Minor</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">21</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ретраи джобов: 2 вместо 3</t>
+          <t>Ретраи джобов: 2 вместо 3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Джоб падает 3 раза.
 Actual Result: failed после 2 ретраев, 1800s никогда.
 Expected Result: 3 ретрая по контракту 8.2.
@@ -789,34 +1090,29 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Major</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Major</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">22</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Антиспам блокирует все включая /start после ~20 действий</t>
+          <t>Антиспам блокирует все включая /start после ~20 действий</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. Активно проходить оформление (клики + тексты + фото).
 2. Набрать &gt;20 апдейтов за минуту.
 Actual Result: 5 минут тишины, /start не оживляет.
@@ -826,34 +1122,29 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">23</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Альбом фото считается как одно: гонка сессии</t>
+          <t>Альбом фото считается как одно: гонка сессии</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">STR:
+          <t>STR:
 1. В checkout.photos отправить альбом из 5 фото разом.
 Actual Result: в черновике оставалось 1 фото (last writer wins при параллельных апдейтах).
 Expected Result: все фото засчитаны.
@@ -862,20 +1153,303 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Critical</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Нет фото после открытия товара на экране товара</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>STR:
+ Будучи клиентом отправить /start;
+ Будучи клиентом нажать «Каталог» → список категорий → список товаров;
+ Открыть любой товар.
+Actual Result: Нет фото после открытия товара на экране товара.
+Expected Result: Есть фото примера товара (example of the product) после открытия товара на экране товара.
+Resolution (FIXED): карточка товара показывает фото (renderProductCard: delete текстового экрана + sendPhoto с подписью и клавиатурой; перерендеры при смене опций идут тем же путём).</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Нет возможности отправить контакт кнопкой при оформлении заказа</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Preconditions: Нужно быть клиентом. Нужен товар в корзине для возможности оформления заказа.
+STR:
+ Нажать кнопку Оформить заказ;
+ Пройти валидно до этапа отправки контакта.
+Actual Result: Нет возможности отправить контакт кнопкой при оформлении заказа.
+Expected Result: Есть возможность отправить свой контакт кнопкой при оформлении заказа на этапе отправки контакта.
+Resolution (FIXED, tech v1.28): шаг контактов присылает reply-клавиатуру с кнопкой «Отправить контакт» (request_contact); транзитное поле SessionData.contactKbMsgId; уборка на всех выходах (контакт/текст/skip/back/cancel//start//menu). Тесты tests/contact-share.test.ts.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>«Пришлите фото или файл чека.», что не соответствует документации tech.md</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Preconditions: Нужно 2 аккаунта, одним быть клиентом, вторым овнером. Нужен уже оформленный товар но не подтвержденный.
+STR:
+ Будучи овнером принять заказ;
+ Будучи клиентом нажать кнопку Я оплатил.
+Actual Result: «Пришлите фото или файл чека.», что не соответствует документации tech.md.
+Expected Result: Пришлите фото чека или тому подобное, без упоминания файла.
+Resolution (ДЕЛО ОТКЛОНЕНО как stated, но underlying contradiction FIXED): tech §9.5 и §8.6 ТРЕБУЮТ приём файлов («фото или файл чека», «оба фото/файл уходят владельцу»). Код раньше врал: промпт обещал файлы, а message:document их отвергал. Исправлено: документы принимаются (handleReceipt document-path), текст invalidReceipt приведён к правде. Если нужен photo-only — это смена контракта (tech v1.2x), скажи, сделаю.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Клиент не может прислать другой чек, так как кнопки «Я оплатил» не приходит.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Preconditions: Нужно 2 аккаунта, одним быть клиентом, вторым овнером. Нужен уже оформленный товар но не подтвержденный.
+STR:
+ Будучи овнером принять заказ;
+ Будучи клиентом нажать кнопку Я оплатил и отправить фото чека;
+ Будучи овнером нажать кнопку «Оплата не пришла».
+Actual Result: Клиент не может прислать другой чек, так как кнопки «Я оплатил» не приходит вместе с сообщением «Оплата не подтверждена. Нажмите «Я оплатил» в сообщении с реквизитами и пришлите другой чек.».
+Expected Result: Клиент может отправить другое фото чека, кнопка «Я оплатил» приходит вместе с сообщением.
+Resolution (FIXED): уведомление badpay идёт с инлайн-кнопкой «Я оплатил» (pay:sent:orderId); notifyCustomer принимает опциональную клавиатуру.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Текст «Оплата не подтверждена. Нажмите «Я оплатил» в сообщении с реквизитами и пришлите другой чек.», не соответствует документации tech.md</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Preconditions: Нужно 2 аккаунта, одним быть клиентом, вторым овнером. Нужен уже оформленный товар но не подтвержденный.
+STR:
+ Будучи овнером принять заказ;
+ Будучи клиентом нажать кнопку Я оплатил и отправить фото чека;
+ Будучи овнером нажать кнопку «Оплата не пришла».
+Actual Result: Текст «Оплата не подтверждена. Нажмите «Я оплатил» в сообщении с реквизитами и пришлите другой чек.», не соответствует документации tech.md.
+Expected Result: В тексте нет упоминания про старое сообщение с реквизитами так как это не соответствует документации tech.md и правилу один экран = одно сообщение. 
+Resolution (FIXED): текст заменён на «❌ Оплата не подтверждена. Пришлите другой чек.» (+кнопка из #27) — без отсылок к старому сообщению, один экран.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>UZ-режим: смесь русского и узбекского по всему боту</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>STR: 1. Переключить магазин на uz (скриптом). 2. Открыть каталог/корзину/оформление/настройки как клиент и владелец.
+Actual Result: десятки захардкоженных русских строк мимо ctx.t (кнопки Отмена/Назад/В меню, карточки заказов, джобы-напоминания, дайджест, статистика, календарь). В ru-режиме незаметно, в uz — каша из двух языков.
+Expected Result: все пользовательские тексты через ctx.t / stringsFor(tenant.language), uz-словарь зеркалит ru.
+Fix: миграция ~100 точек на ctx.t + stringsFor в джобах/notify/digest; localeFor для дат; удалён мёртвый ownerOrders.msg; тесты зелёные без изменения ru-текстов.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>В главном меню нет кнопки «Написать мастеру»</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>STR: 1. Клиент открывает /start. 2. Смотреть кнопки меню.
+Actual Result: только Каталог/Корзина/Мои заказы/FAQ. Кнопки rel:start нет, хотя tech 9.1 требует её в стартовом наборе.
+Expected Result: 5-я кнопка «Написать мастеру» (ctx.t.relay.writeButton) в customerMenuKeyboard.
+Fix: добавлена строка меню + smoke-test.md SMOKE-01 п.1.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Даты форматируются всегда как ru-RU</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>STR: 1. Магазин на uz. 2. Принять заказ с предоплатой, посмотреть срок оплаты и карточку заказа.
+Actual Result: Intl.DateTimeFormat захардкожен на ru-RU в sendPaymentCard, buildOrderCardText/formatDue.
+Expected Result: localeFor(tenant.language) — uz-Latn для uz-магазинов.
+Fix: localeFor в payment-handler и orders.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Экран даты показывает «Лимит: null» при битом оверрайде</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>STR: 1. В capacity_overrides записана строка с capacity NULL. 2. Открыть день в календаре.
+Actual Result: «Лимит: null».
+Expected Result: fallback на defaultDailyCapacity магазина.
+Fix: info.capacity ?? default в showDateScreen + строка через ctx.t.ownerCalendar.limit.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Minor</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(qa): dead keys, dead submit, receipt simplification
Remove unused i18n keys (mirror-checked), wire qrHint and backupCaption. Confirm without draft shows stale hint instead of a dead submit button. Drop unreachable document receipt branches for photo-only contract. Log bug 33.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1449,6 +1449,37 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Мёртвая кнопка «Отправить заказ» при потерянном черновике</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>STR: 1. Начать оформление, дойти до подтверждения. 2. Потерять черновик (сессия сброшена, сообщение осталось). 3. Экран показывает кнопку «Отправить заказ».
+Actual Result: callback chk:submit: (пустой id) не матчится ни одним хендлером — тихая мёртвая кнопка.
+Expected Result: экран staleSubmit без кнопки отправки; пустой submit — no-op без заказа.
+Resolution (FIXED): confirm-ветка показывает staleSubmit без submit-кнопки при отсутствии черновика; тест checkout-steps.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(qa): refresh cases and log bugs 34-38
Fix stale relay/file references, add claim, matrix, kk cases. Log caption overflow, unescaped owner content, silent sticker, dead aboutText.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1478,7 +1478,170 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Фото-карточка падает на длинном описании (caption &gt;1024)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>STR:
+1. Товару задать фото и описание ~2000 символов.
+2. Открыть карточку товара.
+Actual Result: подпись 2040 символов &gt; лимита Telegram 1024 → ошибка API → клиент видит «❌ Произошла ошибка» вместо карточки.
+Expected Result: обрезка подписи с многоточием или fallback на текстовый экран.
+Note QA: воспроизведено зондом P1 (sendPhoto, captionLen 2040, юзеру ушло error-сообщение).</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Экран контактов падает на contactsText &gt;4096</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>STR:
+1. В настройках задать contactsText длиной &gt;4096.
+2. Открыть «📞 Контакты».
+Actual Result: editMessageTextOrSend превышает лимит 4096 → «❌ Произошла ошибка».
+Expected Result: обрезка с многоточием (или лимит длины в валидации настроек).
+Note QA: воспроизведено зондом P2. Тот же класс, что 34: контент владельца без ограничений vs лимиты Telegram.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Контент владельца не экранируется в HTML-сообщениях</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>STR:
+1. Названию магазина задать значение `&lt;b&gt;Hack` (или `&lt;` в greetingText/busyText/paymentText/contactsText).
+2. Открыть /start как клиент.
+Actual Result: сырой `&lt;b&gt;` уходит в HTML-сообщение (доказано зондом P6: greeting содержит «&lt;b&gt;Hack»); на реальном Telegram незакрытый тег роняет парсинг → «❌ Произошла ошибка» на каждый /start. Затронуты: shopName, greetingText, busyText, paymentText, contactsText, replySlaText (start.ts, menu.ts, checkout.ts, cart.ts, payment-handler.ts, contacts.ts, links.ts).
+Expected Result: escapeHtml() вокруг owner-контента по правилу «весь ввод экранируется» (контент владельца — тоже ввод).
+Note QA: пользовательский ввод уже экранируется, пробел только в owner-контенте.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Стикер/голос в ожидании чека игнорируется молча</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>STR:
+1. Дойти до «пришлите фото чека».
+2. Отправить стикер (или голос/видео).
+Actual Result: тишина — ни invalidReceipt, ни реакции (зонд P4). Текст и документы получают подсказку, остальные типы — нет.
+Expected Result: та же подсказка invalidReceipt для любого неподходящего типа.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Настройка «О нас» (aboutText) нигде не показывается</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>STR:
+1. Заполнить «О нас» в настройках.
+2. Искать текст в клиентском боте.
+Actual Result: поле редактируется, но не рендерится ни на одном экране (только грузится в ctx.tenant).
+Expected Result: либо показать (например, в «📞 Контакты» или /start), либо убрать поле из настроек.
+Note QA: найдено код-ревью (render-сайтов aboutText нет).</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): resolutions for bugs 34-38, log bug 33
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -1497,7 +1497,8 @@
 2. Открыть карточку товара.
 Actual Result: подпись 2040 символов &gt; лимита Telegram 1024 → ошибка API → клиент видит «❌ Произошла ошибка» вместо карточки.
 Expected Result: обрезка подписи с многоточием или fallback на текстовый экран.
-Note QA: воспроизведено зондом P1 (sendPhoto, captionLen 2040, юзеру ушло error-сообщение).</t>
+Note QA: воспроизведено зондом P1 (sendPhoto, captionLen 2040, юзеру ушло error-сообщение).
+Resolution (FIXED): подпись фото-карточки обрезается до 1024 через domain/truncateText (без разрыва эмодзи); тест product-photo.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1510,7 +1511,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1530,7 +1530,8 @@
 2. Открыть «📞 Контакты».
 Actual Result: editMessageTextOrSend превышает лимит 4096 → «❌ Произошла ошибка».
 Expected Result: обрезка с многоточием (или лимит длины в валидации настроек).
-Note QA: воспроизведено зондом P2. Тот же класс, что 34: контент владельца без ограничений vs лимиты Telegram.</t>
+Note QA: воспроизведено зондом P2. Тот же класс, что 34: контент владельца без ограничений vs лимиты Telegram.
+Resolution (FIXED): экран контактов обрезается до 4096 через truncateText.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1543,7 +1544,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1563,7 +1563,8 @@
 2. Открыть /start как клиент.
 Actual Result: сырой `&lt;b&gt;` уходит в HTML-сообщение (доказано зондом P6: greeting содержит «&lt;b&gt;Hack»); на реальном Telegram незакрытый тег роняет парсинг → «❌ Произошла ошибка» на каждый /start. Затронуты: shopName, greetingText, busyText, paymentText, contactsText, replySlaText (start.ts, menu.ts, checkout.ts, cart.ts, payment-handler.ts, contacts.ts, links.ts).
 Expected Result: escapeHtml() вокруг owner-контента по правилу «весь ввод экранируется» (контент владельца — тоже ввод).
-Note QA: пользовательский ввод уже экранируется, пробел только в owner-контенте.</t>
+Note QA: пользовательский ввод уже экранируется, пробел только в owner-контенте.
+Resolution (FIXED): escapeHtml() на весь owner-контент (greeting/shopName/busy/payment/contacts/about/replySla/delivery) в start/menu/links/cart/checkout/payment/contacts; доказан зондом P6.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1576,7 +1577,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1595,7 +1595,8 @@
 1. Дойти до «пришлите фото чека».
 2. Отправить стикер (или голос/видео).
 Actual Result: тишина — ни invalidReceipt, ни реакции (зонд P4). Текст и документы получают подсказку, остальные типы — нет.
-Expected Result: та же подсказка invalidReceipt для любого неподходящего типа.</t>
+Expected Result: та же подсказка invalidReceipt для любого неподходящего типа.
+Resolution (FIXED): catch-all на прочие типы сообщений в payment.await_receipt показывает invalidReceipt.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1608,7 +1609,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1628,7 +1628,8 @@
 2. Искать текст в клиентском боте.
 Actual Result: поле редактируется, но не рендерится ни на одном экране (только грузится в ctx.tenant).
 Expected Result: либо показать (например, в «📞 Контакты» или /start), либо убрать поле из настроек.
-Note QA: найдено код-ревью (render-сайтов aboutText нет).</t>
+Note QA: найдено код-ревью (render-сайтов aboutText нет).
+Resolution (FIXED): aboutText показывается в карточке контактов; deliveryText — на шаге адреса.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1641,7 +1642,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log stats bugs 39-41
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1643,6 +1643,99 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Источник «неизвестно» всегда по-русски в статистике</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>STR:
+1. Магазин на uz/kk. 2. Открыть статистику при клиентах без source.
+Actual Result: «• неизвестно: N» по-русски посреди узбекского/казахского экрана (доказано рендером: «Yangi mijozlar: 1 / • неизвестно: 1»). Фолбэк захардкожен в services/stats.ts.
+Expected Result: подпись из словаря (stats.unknownSource) на языке магазина.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>«1 клиентов» — сломанное склонение в статистике</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>STR:
+1. Один просмотр каталога/FAQ без free_text. 2. Открыть статистику.
+Actual Result: «Обрабатывал бот без владельца: 1 клиентов» (и «2 клиентов», «3 клиентов»).
+Expected Result: 1 клиент / 2–4 клиента / 5+ клиентов (в uz/kk существительные не склоняются — там ок).</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Порядок воронки и статусов в статистике случайный</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>STR:
+1. Нагнать события/заказы вперемешку. 2. Открыть статистику.
+Actual Result: шаги воронки и статусы идут в порядке GROUP BY из SQLite (доказано рендером: «Корзина, FAQ, Заказ» и «Отменён, Завершён, Истёк, Чек на проверке»).
+Expected Result: канонический порядок (воронка по стадиям, статусы по жизненному циклу).</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(qa): resolutions for bugs 39-41
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -1659,7 +1659,8 @@
           <t>STR:
 1. Магазин на uz/kk. 2. Открыть статистику при клиентах без source.
 Actual Result: «• неизвестно: N» по-русски посреди узбекского/казахского экрана (доказано рендером: «Yangi mijozlar: 1 / • неизвестно: 1»). Фолбэк захардкожен в services/stats.ts.
-Expected Result: подпись из словаря (stats.unknownSource) на языке магазина.</t>
+Expected Result: подпись из словаря (stats.unknownSource) на языке магазина.
+Resolution (FIXED): сервис возвращает source=null, подпись из словаря (stats.unknownSource ru/uz/kk).</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1672,7 +1673,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1690,7 +1690,8 @@
           <t>STR:
 1. Один просмотр каталога/FAQ без free_text. 2. Открыть статистику.
 Actual Result: «Обрабатывал бот без владельца: 1 клиентов» (и «2 клиентов», «3 клиентов»).
-Expected Result: 1 клиент / 2–4 клиента / 5+ клиентов (в uz/kk существительные не склоняются — там ок).</t>
+Expected Result: 1 клиент / 2–4 клиента / 5+ клиентов (в uz/kk существительные не склоняются — там ок).
+Resolution (FIXED): склонение 1 обращение / 2-4 обращения / 5+ обращений (uz/kk без изменений — не склоняются); заодно «клиентов» → «обращений» по tech §10.8.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1703,7 +1704,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1721,7 +1721,8 @@
           <t>STR:
 1. Нагнать события/заказы вперемешку. 2. Открыть статистику.
 Actual Result: шаги воронки и статусы идут в порядке GROUP BY из SQLite (доказано рендером: «Корзина, FAQ, Заказ» и «Отменён, Завершён, Истёк, Чек на проверке»).
-Expected Result: канонический порядок (воронка по стадиям, статусы по жизненному циклу).</t>
+Expected Result: канонический порядок (воронка по стадиям, статусы по жизненному циклу).
+Resolution (FIXED): канонический порядок воронки и статусов в хендлере; мёртвый free_text скрыт из воронки (в подсчёте участвует).</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1734,7 +1735,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log presale bugs 42-44
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1736,6 +1736,102 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Пустой магазин показывает грубое «Категории не найдены»</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>STR:
+1. Новый магазин без категорий. 2. Открыть каталог клиентом.
+Actual Result: «🔍 Категории не найдены.», а дружелюбный catalog.empty («В магазине пока нет категорий») нигде не используется — мёртвый ключ.
+Expected Result: пустой магазин показывает catalog.empty.
+Resolution (FIXED): cat:list использует catalog.empty; categoriesEmpty остался для пропавшей категории.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SLA по умолчанию всегда по-русски в uz/kk-магазинах</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>STR:
+1. Новый магазин на uz/kk без своих текстов. 2. Оформить заказ.
+Actual Result: «... Шебер жауап береді в течение нескольких часов» — replySlaText единственный owner-текст без dict-fallback (NOT NULL + русский дефолт).
+Expected Result: стоковый дефолт читается как «не задано», подставляется orderSentSlaDefault на языке магазина.
+Resolution (FIXED): сравнение со STOCK_RU_SLA в checkout + ключи orderSentSlaDefault ×3.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Демо-сид полностью на английском</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>STR:
+1. Запустить npm run seed. 2. Открыть демо-бота.
+Actual Result: весь демо-контент (магазин, каталог, FAQ) на английском — стыдно показывать RU-клиентам. Плюс seed.ts искал товары по названиям (хрупко для переводов).
+Expected Result: русский демо-контент; привязка опций по стабильным titleKey.
+Resolution (FIXED): переведены tenant/categories/products/options/faq; productMap по titleKey; обновлены 3 ассёрта.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(onescreen): edit everywhere instead of new messages
Root cause: ownerDraft (with screen id) was cleared before rendering, so every settings/catalog/FAQ save sent a new message. Thread the draft through. Same audit pass: busy/paused/pay errors edit the screen, QR view removes the list first, pd:yes drops the redundant notice. Bug 45.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1766,7 +1766,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1798,7 +1797,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1830,7 +1828,38 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Сохранение настройки создаёт новое сообщение вместо правки экрана</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>STR:
+1. Владелец открывает Настройки → любое поле → вводит значение.
+Actual Result: каждое сохранение слало НОВОЕ сообщение (чат плодился). Корень: хендлер чистил ownerDraft (со screen id) ДО отрисовки результата, editScreenOrSend не находил экран и уходил в sendMessage-ветку.
+Expected Result: один экран — правка промпта (tech §9).
+Resolution (FIXED): screen id проброшен через draft-объект во все вызовы; регрессионный тест в settings.test.ts. Попутно по аудиту всех кнопок: busy/paused/pay-ошибки и QR теперь тоже правят/чистят экран вместо новых сообщений; убран лишний дабл-нотифай в pd:yes.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(contracts): v1.35 closed-date toasts, option All-query
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1859,7 +1859,38 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Скрытую опцию нельзя включить обратно (и её не видно в списке)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>STR:
+1. Владелец скрывает опцию товара. 2. Пытается включить обратно.
+Actual Result: showOptionList и opttoggle используют listProductOptions (только isActive), скрытая опция пропадает из списка и toggle молча no-op.
+Expected Result: список показывает все опции с меткой 🙈, toggle работает в обе стороны.
+Resolution (FIXED): listProductOptionsAll в services/catalog.ts; tech v1.35.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(cart): hidden products rejected with honest toast
prd:add used the unfiltered lookup, so stale cards added invisible products while toasting success. Now getProductIfOwned with a not-found toast. Bug 47.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1890,7 +1890,38 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Скрытый товар добавляется в корзину с тостом «Добавлено»</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>STR:
+1. Владелец скрывает товар. 2. Клиент жмёт «В корзину» на старом экране карточки.
+Actual Result: prd:add брал getProductById (без проверки активности), тост «✅ Добавлено» врал, строка падала в корзину (позже submit отклонял с productInactive).
+Expected Result: скрытый/удалённый товар не добавляется, тост «Товар не найден».
+Resolution (FIXED): getProductIfOwned + честный тост; тест в cart.test.ts.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(cards): photo render fallback, honest add toast
Any sendPhoto failure falls back to the text card instead of erroring every interaction. Bug 48.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1921,7 +1921,38 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Любой сбой отправки фото роняет всю карточку товара</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>STR:
+1. Товар с битым/протухшим photoFileId (или подписью за лимитом на живом API). 2. Открыть карточку / ткнуть опцию.
+Actual Result: sendPhoto бросал исключение наружу → error-middleware показывал «❌ Произошла ошибка» на каждое действие с карточкой; выбор выглядел «застрявшим».
+Expected Result: fallback на текстовую карточку, пользователь ошибки не видит.
+Resolution (FIXED): send-first-then-delete + catch с fallback на текст; тест с инжектом ошибки.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(links): validate source labels
Empty and overlong labels now rejected with badLabel like other editors. Bug 49.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1952,7 +1952,68 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Пустая и слишком длинная source-метка принимаются</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>STR:
+1. Владелец: ссылки → новая метка. 2. Отправить пустой текст или 200 символов.
+Actual Result: обе приняты (пустая получила авто-код src_xxxxxx), badLabel-кнопка нигде не использовалась.
+Expected Result: отклонение с «Название не подходит», как у категорий.
+Resolution (FIXED): валидация 1..64 в src_add_label + тест.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Нет предупреждения, когда настройки гасят все даты</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>STR:
+1. Поставить minLeadDays 90 при maxAdvance 60 (или лимит 0). 2. Открыть оформление.
+Actual Result: весь календарь ✕ без единого слова владельцу — он уверен, что «всё открыто» (календарь показывает лимиты). Код формально прав (TOO_SOON/FULL), UX нет.
+Expected Result: предупреждение владельцу (тост/строка в календаре) при нуле доступных дат; зонд: LEAD90 0/28, CAP0 0/28.
+Note QA: НЕ исправлено, ждёт решения — вариант: строка-предупреждение на экране даты владельца.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(settings): warn when settings close all dates
Static check on the settings list: minLeadDays > maxAdvanceDays or defaultDailyCapacity < 1 closes every date, so the screen shows a warning line. Texts in ru/uz/kk, probed with zero-available cases. Bug 50.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -2014,6 +2014,11 @@
           <t>Minor</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Resolution (FIXED): экран настроек теперь показывает статичные предупреждения при minLeadDays &gt; maxAdvanceDays и defaultDailyCapacity &lt; 1 (оба случая гасят все даты). Тест в settings.test.ts.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(bot): harden dates, cancel scoping, delete UX
Bug 51: strict isValidIsoDate/isValidIsoMonth + guards in 10 handlers (crafted 9999-99-99 no longer pings superadmin). Bug 52: my:cancel checks order ownership. Bug 53: HAS_PRODUCTS explains via alert. Bug 54: product delete is two-step (adm:prd:delcf, codec + tech.md v1.37). Tests: qa-fixes.test.ts (7).
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2020,6 +2020,134 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Невозможные даты в callback/`9999-99-99` роняют хендлеры</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>STR:
+1. Отправить боту callback chk:date:9999-99-99 (или chk:closed / chk:datepage:9999-99 / adm:cal:day / toggle / setcap / page, adm:ord:datepage / pd с битой датой).
+Actual Result: RangeError Invalid time value, пользователю — общая ошибка, суперадмину — пинг «Ошибка бота» (4 пинга на 8 колбэков). Любой пользователь может спамить суперадмина крафт-колбэками.
+Expected Result: молчаливый игнор после answerCallback.
+Resolution (FIXED): строгие isValidIsoDate/isValidIsoMonth в lib/time.ts + гарды в 10 местах (checkout x3, calendar x4, orders x2... datepage+pd). Тест bug 51: 0 пингов.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Экран причин отмены показывался для чужого заказа</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>STR:
+1. my:cancel:&lt;чужой orderId&gt; от другого клиента.
+Actual Result: показывался список причин отмены (финальная отмена проверяла владение — doCustomerCancel, данные в безопасности).
+Expected Result: «Заказ не найден» как в my:view.
+Resolution (FIXED): ownership-lookup в my:cancel + тест bug 52.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Удаление непустой категории молча ничего не делало</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>STR:
+1. Владелец: категория с товарами → Удалить.
+Actual Result: список молча перерисовывался, обе ветки if/else делали одно и то же, причина HAS_PRODUCTS нигде не объяснялась.
+Expected Result: объяснение.
+Resolution (FIXED): алерт ownerCatalog.catNotEmpty (ru/uz/kk) + тест bug 53.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Удаление товара — один тап без подтверждения</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>STR:
+1. Владелец: товар → Удалить.
+Actual Result: товар + все опции уничтожались одним тапом, без undo.
+Expected Result: подтверждение.
+Resolution (FIXED): два шага adm:prd:del → экран-подтверждение → adm:prd:delcf (кодек + tech.md v1.37). Тест bug 54.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(load): flash-sale 50 clients for 30 slots
50 simultaneous full UI checkouts on one date: asserts slots exactly filled (no oversell), losers honestly rejected, zero crashes, no duplicate idempotency keys.
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2050,7 +2050,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2082,7 +2081,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2114,7 +2112,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2146,7 +2143,42 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Языковой проход uz/kk: кальки, порядок слов, эмодзи</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Автоматический аудит 363 ключей (совпадения с ru, баланс HTML, арность, эмодзи) + ручная вычитка.
+Найдено и исправлено:
+- kk «профиль қалпақшасы» x3 → «профиль сипаттамасы» (калька с русского).
+- kk «Бүгін мен ертең» → «Бүгін және ертең» (неверный союз).
+- kk пример группы опций «Салма» (вес) → «Салмасы» (начинка).
+- uz backupCaption «MB dayjesti» → «MB nusxasi» (дайджест вместо бэкапа).
+- uz/kk orderSent SOV-порядок: «...javob beradi bir necha soat ichida» → SLA по умолчанию в скобках.
+- kk два empty-состояния без эмодзи (🔗📋).
+Совпадения с ru в kk («Каталог», «Клиент», «Валюта» и т.п.) — корректные заимствования, не баги.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bugs 56-57
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2178,7 +2178,67 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Упавший поллинг одного бота ронял весь процесс</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>STR:
+1. Токен одного магазина отозван (401) или запущен второй процесс с тем же токеном (409) во время работы.
+Actual Result: задача раннера реджектилась, handle.task() никто не наблюдал → unhandled rejection → падение ВСЕГО процесса со всеми магазинами. Нарушение «ошибка одного бота не останавливает остальные».
+Expected Result: изоляция + уведомление суперадмина.
+Resolution (FIXED): watchTask/onTenantDown в runner.ts: 401/409 — снять тенант + уведомить, без рестарта; прочие — уведомить + рестарт опроса через минуту (stopTenant отменяет). Тест runner.test.ts (4). tech.md v1.38.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Тон клиентских текстов: сухо, тупики без CTA</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Проход глазами: приветствие сухое («Приятно познакомиться»), пустые корзины/заказы/категории — тупики без призыва, отмена мастером и busy без эмпатии/альтернативы, реквизиты — обрывком.
+Resolution (FIXED): тёплое приветствие с CTA в каталог, CTA в пустых состояниях, «спасибо» в orderSent, эмпатия в cancelledByOwner + указание на Контакты, busy и noRequisites с направлением в Контакты. Зеркально в uz/kk.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bugs 58-60
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2209,7 +2209,6 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2238,7 +2237,99 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>/resume с упавшим стартом оставлял фантомно-активный магазин</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>STR:
+1. Магазин на паузе. 2. /resume demo при битом токене (startTenant бросает).
+Actual Result: статус в БД уже переключён на active, исключение уходило в общий error-хендлер, бот мёртв, суперадмин видит только generic error. Магазин «активен», но не работает.
+Expected Result: откат на paused + понятная ошибка.
+Resolution (FIXED): try/catch вокруг startTenant с revert на paused и текстом реальной причины. Тест bug 58.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>chk:photos:done перепрыгивал из любого состояния сразу в confirm</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>STR:
+1. Застрять на шаге комментария (например, 501 символ отклонён). 2. Прислать chk:photos:done.
+Actual Result: безусловный переход в checkout.confirm, пропуск шагов. Через UI недостижимо (кнопки нет), только крафт.
+Expected Result: игнор вне checkout.photos.
+Resolution (FIXED): guard на состояние + тест bug 59.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Нет лимитов длин и верхних границ чисел (против tech §12)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Tech требует «ограничения на ввод: длины текстовых полей, валидация телефона», но: время/адрес/имя клиента без кэпов (4000 символов → экран &gt;4096 → 400 у Telegram), телефон принимал «++-----» (цифры не требовались), minLead/maxAdvance/deadline/capacity/deliveryFee и цена товара без верхних границ (торт за 1 трлн ₽).
+Resolution (FIXED): время ≤100, адрес ≤500, имя ≤100 (common.badText), телефон: charset + ≥7 цифр + ≤25 символов; дни ≤3650, capacity ≤10000, деньги ≤9 999 999 999 minor (digit-cap — minor unit различаются по валютам); цена товара через тот же кэп (badPrice). Тесты bug 60.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bugs 61-62
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2268,7 +2268,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2300,7 +2299,6 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2329,7 +2327,70 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Джобы двоились при двух процессах (нет claim)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>STR:
+1. Запустить два шедулера (два процесса с одним токеном/БД, сценарий 409). 2. Дождаться тика.
+Actual Result: оба забирали одни и те же pending-джобы — доказано тестом: 4 исполнения вместо 1-2. Клиенты получали дубли напоминаний/дайджестов.
+Expected Result: ровно одно исполнение.
+Resolution (FIXED): атомарный claim одним UPDATE ... WHERE status='pending' (проигравший пропускает), статус running в схеме, лиза 10 минут + reaper упавших воркеров (crash засчитывается как попытка). 0007_job_claim.sql — no-op (SQLite не материализует text-enum). tech.md v1.39. По пути удалён битый 0003_short_lorna_dane.sql от drizzle-kit (перегенерированная старь, роняла бы migrate на чистой БД) и откачены мусорные meta-правки.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Битый tenant.timezone ронял все экраны дат</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>STR:
+1. Поставить tenants.timezone='Mars/Olympus' (прямая правка БД). 2. Открыть оформление/календарь.
+Actual Result: Intl.DateTimeFormat бросал RangeError на каждом рендере дат — checkout и календарь мертвы, суперадмину пинг за каждый показ.
+Expected Result: работа с фолбэком.
+Resolution (FIXED): safeTimeZone в lib/time.ts (toIsoDate + zonedTimeToUtc): фолбэк на UTC + console.error. Тест bug 61.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bug 63
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2358,7 +2358,6 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2390,7 +2389,38 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Старые заказы показывали новую валюту после переключения</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>STR:
+1. Заказ в ₽. 2. Настройки → валюта ₸. 3. Открыть старый заказ.
+Actual Result: суммы в minor без изменений, но с новым символом (1400₽ → «1 400 ₸»).
+Expected Result: символ на момент создания.
+Resolution (FIXED): снимок orders.currency при создании (backfill из tenants в 0008), карточка/контакты/чеки используют order.currency. tech.md v1.40. Агрегаты статистики после смены валюты по-прежнему смешивают символы — принято как есть (редкий кейс настройки).</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bug 64
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2420,7 +2420,38 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Claim-код срабатывал из чужого бота (передача владения)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>STR:
+1. Взять claim-ссылку магазина A. 2. Вручную отправить /start claim_&lt;код-A&gt; в чат с ботом магазина B (тот же процесс).
+Actual Result: claimTenant искал код по хешу глобально → владелец B становился владельцем A. Эскалация через набранную вручную команду.
+Expected Result: код действителен только в своём боте.
+Resolution (FIXED): claimTenant принимает tenantId, поиск по паре (хеш, tenant); чужая попытка возвращает NOT_FOUND и код не сжигает (проверено: код после работает в своём боте). tech.md v1.41. Изоляция остального (заказы/корзины/сессии/роли) проверена честным двухтенантным тестом — чисто.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bug 65
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2451,7 +2451,38 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Удаление тенанта не чистило feature_flags</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>STR:
+1. Выставить магазину флаг (напр. daily_digest off). 2. Удалить тенант через tenant:delete.
+Actual Result: строки feature_flags оставались сиротами; при пересоздании того же слага магазин наследовал чужие флаги.
+Expected Result: полное удаление.
+Resolution (FIXED): DELETE FROM feature_flags в транзакции + тест. Сверены все 16 таблиц со схемой — остальное чистится.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bugs 66-67
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2482,7 +2482,70 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Заказы за пределами 8 в группе не открывались никак</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>STR:
+1. Создать 25 новых заказов. 2. adm:ord:list.
+Actual Result: показаны 8, остальные 17 без кнопки «ещё» — недоступны из UI вообще.
+Expected Result: листание.
+Resolution (FIXED): adm:ord:more:&lt;group&gt;:&lt;page&gt; (кодек + таблица колбэков), по 8 на страницу, лимит выборки 50→200. tech.md v1.42. Тест bug 66 (8→16→24→25).</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>PDF принимался как фото товара</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>STR:
+1. Товар → поле фото → прислать PDF-документ.
+Actual Result: file_id документа сохранялся в photoFileId + «Сохранено» — карточка падала на показе (sendPhoto с file_id документа).
+Expected Result: отказ с подсказкой.
+Resolution (FIXED): ветка document показывает ownerCatalog.badPhoto (ru/uz/kk), черновик и состояние сохраняются — следующее фото принимается. Тест bug 67.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bug 68
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2513,7 +2513,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2545,7 +2544,38 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Поддельный код причины отмены сохранялся как есть</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>STR:
+1. my:cancelreason:&lt;свой orderId&gt;:injected (крафт-колбэк).
+Actual Result: произвольный текст падал в orders.cancelReason и показывался владельцу (хендлер принимал любой [a-z]+ мимо кодека).
+Expected Result: только контрактные коды.
+Resolution (FIXED): fallback на cancelReasons.other. Контрактный аудит: схема БД == tech §5 по всем 16 таблицам (автосверка); все хендлеры отвечают answerCallback; комментарий language в §5 поправлен (ru|uz|kk).</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bug 69
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2575,7 +2575,38 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Срок/лимит товара и лимит дня без верхних границ</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>STR:
+1. Товар → поле срока → 999999999 (или лимит 999999999).
+Actual Result: принималось (срок 999M дней = товар-мёртвый, тихий отказ всем датам). Настройки-числа были capped в bug 60, товарные/календарные — нет.
+Expected Result: отказ.
+Resolution (FIXED): lead ≤3650, capacity/cal_capacity ≤10000, тем же badNumber/badCapacity. Тест bug 69.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bugs 70-72
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2606,7 +2606,100 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Обрезка подписи рвала HTML (400 от Telegram)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>STR:
+1. Товар с фото + описание ~1000 символов с &amp; &lt; &gt; так, чтобы граница 1024 легла внутрь сущности/тега.
+Actual Result: truncateText резал вслепую → &amp;am… / &lt;b… → sendPhoto с parse_mode HTML падал 400, клиент видел общую ошибку.
+Expected Result: аккуратная обрезка.
+Resolution (FIXED): truncateHtml (не рвёт теги/сущности, закрывает открытые, plain-фолбэк) + unit/property-тесты. Применён в карточке товара.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Дайджест ломался на 200+ заказах в день</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>STR: 55+ заказов на дату → текст &gt;4096.
+Actual Result: sendMessage 400 → джоб в ретраи, в пик сезона дайджеста нет.
+Expected Result: влезать всегда.
+Resolution (FIXED): строки режутся по 20/день с пометкой digestMore (ru/uz/kk); кнопки и так были 10. Тест bug 71.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Свой список заказов без пагинации (кнопок &gt;100 = 400)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>STR: 100+ заказов у клиента → клавиатура сверх лимита Telegram.
+Actual Result: потенциальный 400 (редкий кейс постоянных клиентов).
+Expected Result: листание.
+Resolution (FIXED): my:more:&lt;page&gt; по 10 (кодек + таблица), зеркало owner-паттерна. Тест bug 72 (10→12). Каталоги/FAQ/редакторы оставлены как есть (реалистично &lt;100 позиций, владелец контролирует размер) — зафиксировано как известный предел.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): log bug 73
</commit_message>
<xml_diff>
--- a/docs/qa/bugs.xlsx
+++ b/docs/qa/bugs.xlsx
@@ -408,7 +408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2637,7 +2637,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2668,7 +2667,6 @@
           <t>Major</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2699,7 +2697,38 @@
           <t>Minor</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Правка удалённой цели врала «Сохранено»</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>STR:
+1. Открыть редактирование товара/категории/вопроса. 2. Удалить цель (вторая сессия). 3. Отправить текст.
+Actual Result: «✅ Сохранено», хотя писать некуда (UPDATE по нулю строк).
+Expected Result: честное «не найдено».
+Resolution (FIXED): updateCategoryTitle/updateProduct/updateFaq возвращают boolean (RETURNING); хендлеры показывают notFound (catNotFound новый ключ ru/uz/kk, product/faq существующие). Тест bug 73 (все три цели).</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>